<commit_message>
chore: regenerate manifest xlsx workbooks
</commit_message>
<xml_diff>
--- a/excel_templates/methylation_manifest_template.xlsx
+++ b/excel_templates/methylation_manifest_template.xlsx
@@ -497,7 +497,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PT1899</t>
+          <t>P_5P2QIUH2</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>SM7316-11566</t>
+          <t>S_0000012</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AL1549608_T_WGS</t>
+          <t>AL_0000025_T_Methyl</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>MODEL-PARENT-001</t>
+          <t>CNMC-XD760</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>MODEL-GM-001</t>
+          <t>CNMC-XD760-mCherry-Luciferase</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>impact trial</t>
+          <t>RBT</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">

</xml_diff>